<commit_message>
Drop service-account key mapping; structure GPU unit mapping fields
- Consumer identification no longer collects API key mappings anywhere
  (sheet item removed, serviceAccounts dropped from API and OpenAPI):
  platforms record the consumer's service name at key issuance and
  report usage keyed by that name; unregistered names hit the existing
  alert loop. Items renumbered to [1]-[5]
- gpuDashboardUnits changed from packed prefix strings to structured
  entries (infraType/workgroup/optional unit — empty unit means whole
  workgroup); spec examples, field table, summary, and Excel template
  updated. Recorded as decision 20

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8dM4fn77VhwFZW3VhfGwv
</commit_message>
<xml_diff>
--- a/docs/METADATA_SHEET_TEMPLATE.xlsx
+++ b/docs/METADATA_SHEET_TEMPLATE.xlsx
@@ -12,7 +12,6 @@
     <sheet name="모델" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="GPU할당매핑" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="소비관계" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="서비스계정" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -489,7 +488,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>이 양식은 구현 스펙(docs/METRICS_COLLECTION_SPEC.md) §1의 제출 항목 [1]~[6]을 시트로 나눈 것입니다.</t>
+          <t>이 양식은 구현 스펙(docs/METRICS_COLLECTION_SPEC.md) §1의 제출 항목 [1]~[5]를 시트로 나눈 것입니다.</t>
         </is>
       </c>
     </row>
@@ -513,7 +512,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. 서비스        [1][6] 서비스 표기·담당자 + /metrics URL·엔진 종류 (서비스당 1행)</t>
+          <t xml:space="preserve">  1. 서비스        [1][5] 서비스 표기·담당자 + /metrics URL·엔진 종류 (서비스당 1행)</t>
         </is>
       </c>
     </row>
@@ -527,7 +526,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. GPU할당매핑   [3] GPU 대시보드 할당 unit 프리픽스 목록 (프리픽스당 1행)</t>
+          <t xml:space="preserve">  3. GPU할당매핑   [3] GPU 대시보드 할당 unit 매핑 — unit을 비우면 워크그룹 전체</t>
         </is>
       </c>
     </row>
@@ -539,62 +538,69 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  5. 서비스계정    [5] 플랫폼 제공자만 — 발급한 API 키 ↔ 소비 서비스</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>작성 원칙:</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>작성 원칙:</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · serviceGroup·service·model은 기존 토큰 API(/v1/usage)와 같은 문자열이어야 합니다 (JOIN 조건).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · serviceGroup·service·model은 기존 토큰 API(/v1/usage)와 같은 문자열이어야 합니다 (JOIN 조건).</t>
+          <t xml:space="preserve">  · 모델 canonical 정의(family·paramsB·aliases)는 서빙 주체만 작성 — 사내 플랫폼 경유 모델은 canonical 이름만.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 모델 canonical 정의(family·paramsB·aliases)는 서빙 주체만 작성 — 사내 플랫폼 경유 모델은 canonical 이름만.</t>
+          <t xml:space="preserve">  · 사내 파인튜닝 모델은 반드시 -ft-{용도} 접미로 순정과 분리. 애매하면 나눕니다.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 사내 파인튜닝 모델은 반드시 -ft-{용도} 접미로 순정과 분리. 애매하면 나눕니다.</t>
+          <t xml:space="preserve">  · 플랫폼 제공자는 API 키 매핑을 제출하지 않습니다 — 키 발급 시 소비 서비스의 service 표기를 받아 기록하고,</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 제출 후 갱신은 알림 기반입니다 — 미등록 모델·엔진 교체·검증 위반은 운영자가 감지해 owner에게 알립니다.</t>
+          <t xml:space="preserve">    토큰 사용량 제공 시 소비자 호출분을 그 표기로 구분합니다.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t xml:space="preserve">  · 제출 후 갱신은 알림 기반입니다 — 미등록 모델·엔진 교체·검증 위반은 운영자가 감지해 owner에게 알립니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t xml:space="preserve">  · 엔진 버전은 API(engine 필드) 자기신고로 수신하므로 수기 갱신이 필요 없습니다.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>문의: 토큰 대시보드 운영자 · 상세 규칙: docs/METRICS_COLLECTION_SPEC.md</t>
         </is>
@@ -642,13 +648,13 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>[6] 케이스 A~C만: 스크랩 대상 /metrics URL(VIP)
+          <t>[5] 케이스 A~C만: 스크랩 대상 /metrics URL(VIP)
 해당 없으면 비움</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>[6] 엔진 종류 (vllm/sglang/custom 등)
+          <t>[5] 엔진 종류 (vllm/sglang/custom 등)
 버전은 API 자기신고</t>
         </is>
       </c>
@@ -966,23 +972,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="55" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>소속 서비스 표기</t>
+          <t>소속 서비스 표기
+(GPU 할당 없으면 이 시트에 행 없음)</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>[3] GPU 대시보드 할당 unit 프리픽스 — 인프라유형:워크그룹:unit이름 계층의 어느 수준이든 가능
-워크그룹 수준 권장(하위 unit 자동 포함), 공유 워크그룹만 unit 수준. GPU 할당 없으면 이 시트에 행 없음</t>
+          <t>[3] GPU가 올라간 인프라 유형</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>[3] GPU 대시보드의 워크그룹 이름</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>[3] unit 이름 — **비우면 워크그룹 전체** (권장, 하위 unit 자동 포함)
+워크그룹을 타 서비스와 공유할 때만 지정</t>
         </is>
       </c>
     </row>
@@ -994,7 +1013,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>prefix</t>
+          <t>infraType</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>workgroup</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>unit</t>
         </is>
       </c>
     </row>
@@ -1006,9 +1035,15 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>ai-platform:ds-assistant</t>
-        </is>
-      </c>
+          <t>ai-platform</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>ds-assistant</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1018,9 +1053,15 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>ds-cloud:ds-assistant-batch</t>
-        </is>
-      </c>
+          <t>ds-cloud</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>ds-assistant-batch</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1030,7 +1071,17 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>ds-cloud:search-team:doc-summary-prod</t>
+          <t>ds-cloud</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>search-team</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>doc-summary-prod</t>
         </is>
       </c>
     </row>
@@ -1174,92 +1225,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="55" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>플랫폼 제공자의 서비스 표기</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>[5] 발급한 API 키(서비스 계정) 식별자</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>그 키를 쓰는 소비 서비스의 service 표기
-(API의 serviceAccounts 자기신고로 대체 가능)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>service</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>serviceAccount</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>consumerService</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>ds-assistant-portal</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>svc-key-a1</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>hr-chatbot</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>ds-assistant-portal</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>svc-key-b2</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>doc-summary</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>